<commit_message>
Added new files base, pom, dataprovider etc
</commit_message>
<xml_diff>
--- a/src/main/resources/DDT/Data.xlsx
+++ b/src/main/resources/DDT/Data.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\shashank\Capgemini_Training\Selenium\Adv_Selenium\selenium-advance\src\main\resources\DDT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B63B0BF4-C0ED-4230-8BCD-882FBEEFCFFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A1A00EE-1873-4B22-9A2B-ECC60BB68576}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{77F40206-6188-46F7-88A0-A32B0F7E3BF9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="1" xr2:uid="{77F40206-6188-46F7-88A0-A32B0F7E3BF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>browser</t>
   </si>
@@ -49,6 +50,27 @@
   </si>
   <si>
     <t>secret_sauce</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>shank</t>
+  </si>
+  <si>
+    <t>shashank</t>
+  </si>
+  <si>
+    <t>xxx</t>
+  </si>
+  <si>
+    <t>abc</t>
+  </si>
+  <si>
+    <t>def</t>
+  </si>
+  <si>
+    <t>ijk</t>
   </si>
 </sst>
 </file>
@@ -449,4 +471,50 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{08850874-F6E3-453C-81F6-18147E19AC04}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24.44140625" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>